<commit_message>
Fix duplicate hardware lines in import file
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019oxoH766RXuqLqXQEjeJHj
</commit_message>
<xml_diff>
--- a/Importacao_Lista_de_materiais_04.01.3.000598.xlsx
+++ b/Importacao_Lista_de_materiais_04.01.3.000598.xlsx
@@ -4492,7 +4492,7 @@
         </is>
       </c>
       <c r="C163" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="D163" t="inlineStr">
         <is>
@@ -5010,7 +5010,7 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>Motivo</t>
+          <t>Situação</t>
         </is>
       </c>
     </row>
@@ -5022,12 +5022,12 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>[DEFINIR] PENDENTE: balões 52, 62, 65 sem linha na lista do desenho</t>
+          <t>balões 52, 62, 65 sem linha na lista do desenho</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Sem código/descrição definida</t>
+          <t>A definir (sem código/descrição)</t>
         </is>
       </c>
     </row>
@@ -5039,12 +5039,12 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>[DEFINIR] PENDENTE: desenho 022-007345 (barra superior da alavanca) sem desenho</t>
+          <t>desenho 022-007345 (barra superior da alavanca) sem desenho</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Sem código/descrição definida</t>
+          <t>A definir (sem código/descrição)</t>
         </is>
       </c>
     </row>

</xml_diff>